<commit_message>
chore: commit SM/CP capture scripts, result JSONs, xlsx + report updates
SM capture scripts + result logs: capture-sm-4modules, fix-v2, login-v3
CP capture scripts + result logs: capture-cp-4modules, v2, leads-actions-v3
Updated: TestCases-AdminPortal.xlsx, execution-report (sprint-5 html+xlsx), visual-memory/INDEX.md

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/manual-qa-repository/06-test-runs/UAT/sprint-5/execution-report.xlsx
+++ b/manual-qa-repository/06-test-runs/UAT/sprint-5/execution-report.xlsx
@@ -8884,7 +8884,8 @@
     <t>PASS</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-05-31 19:01 · PASS
+    <t xml:space="preserve">2026-05-31 19:19 · PASS
+2026-05-31 19:01 · PASS
 2026-05-31 19:01 · PASS</t>
   </si>
   <si>
@@ -10418,7 +10419,7 @@
     <t>Generated</t>
   </si>
   <si>
-    <t>2026-05-31 19:01</t>
+    <t>2026-05-31 19:19</t>
   </si>
   <si>
     <t>Sprint</t>

</xml_diff>